<commit_message>
feat: add scraped data for user "还是叫吴富贵吧"
Add five new notes scraped from Xiaohongshu for user "还是叫吴富贵吧".
Each note includes image files, detail.txt metadata, and info.json structured data.
The scraped_urls.txt file is updated with the corresponding URLs.
</commit_message>
<xml_diff>
--- a/datas/excel_datas/5b6150c56b58b741e26b8c7f.xlsx
+++ b/datas/excel_datas/5b6150c56b58b741e26b8c7f.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T666"/>
+  <dimension ref="A1:T671"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -69209,6 +69209,545 @@
         </is>
       </c>
     </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>69462cb0000000001b0250e2</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>https://www.xiaohongshu.com/explore/69462cb0000000001b0250e2?xsec_token=ABfAKOv9KzAlnD02ddaivXvWpZ0WwLhDXjPe2BwC8skmk=&amp;xsec_source=pc_user</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>图集</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>5b6150c56b58b741e26b8c7f</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>https://www.xiaohongshu.com/user/profile/5b6150c56b58b741e26b8c7f</t>
+        </is>
+      </c>
+      <c r="F667" t="inlineStr">
+        <is>
+          <t>还是叫吴富贵吧</t>
+        </is>
+      </c>
+      <c r="G667" t="inlineStr">
+        <is>
+          <t>https://sns-avatar-qc.xhscdn.com/avatar/1040g2jo31g9vkplp2s6g4a7r1e8cb33vdvgmpr0</t>
+        </is>
+      </c>
+      <c r="H667" t="inlineStr">
+        <is>
+          <t>简单点</t>
+        </is>
+      </c>
+      <c r="I667" t="inlineStr">
+        <is>
+          <t>我平安姑娘A20％
+平安姑娘tvb10％
+那么≈30％
+格局掉10％tvb后
+30％≈格局掉了3/1了
+#我的炒股日记[话题]#</t>
+        </is>
+      </c>
+      <c r="J667" t="inlineStr">
+        <is>
+          <t>2081</t>
+        </is>
+      </c>
+      <c r="K667" t="inlineStr">
+        <is>
+          <t>129</t>
+        </is>
+      </c>
+      <c r="L667" t="inlineStr">
+        <is>
+          <t>282</t>
+        </is>
+      </c>
+      <c r="M667" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="N667" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="O667" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="P667" t="inlineStr">
+        <is>
+          <t>['http://sns-webpic-qc.xhscdn.com/202602112034/8fe06beda8f2124ec05f7c1184e89cd3/1040g00831qa6dv9pga5g4a7r1e8cb33vk4vb088!nd_dft_wlteh_jpg_3']</t>
+        </is>
+      </c>
+      <c r="Q667" t="inlineStr">
+        <is>
+          <t>['我的炒股日记']</t>
+        </is>
+      </c>
+      <c r="R667" t="inlineStr">
+        <is>
+          <t>2025-12-20 12:57:20</t>
+        </is>
+      </c>
+      <c r="S667" t="inlineStr">
+        <is>
+          <t>未知</t>
+        </is>
+      </c>
+      <c r="T667" t="inlineStr">
+        <is>
+          <t>图1: OCR超时</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>694626a1000000001b023e32</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>https://www.xiaohongshu.com/explore/694626a1000000001b023e32?xsec_token=ABfAKOv9KzAlnD02ddaivXvRS0LXe637eBtwvvKrDCVUo=&amp;xsec_source=pc_user</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>图集</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>5b6150c56b58b741e26b8c7f</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>https://www.xiaohongshu.com/user/profile/5b6150c56b58b741e26b8c7f</t>
+        </is>
+      </c>
+      <c r="F668" t="inlineStr">
+        <is>
+          <t>还是叫吴富贵吧</t>
+        </is>
+      </c>
+      <c r="G668" t="inlineStr">
+        <is>
+          <t>https://sns-avatar-qc.xhscdn.com/avatar/1040g2jo31g9vkplp2s6g4a7r1e8cb33vdvgmpr0</t>
+        </is>
+      </c>
+      <c r="H668" t="inlineStr">
+        <is>
+          <t>无标题</t>
+        </is>
+      </c>
+      <c r="I668" t="inlineStr">
+        <is>
+          <t>很多事真的不必勉强
+认知 资源 决定以后结果
+变异电是需要用以后来兑现的
+so 我认为好 但依然不推荐
+很多人下面也别唧唧歪歪
+你照照镜子 没人硬塞给你
+你是谁 其实我根本不认识你
+所以不要搞的像真的一样
+一句句为什么 一句句要我分析
+我分析给毛线给你听要么</t>
+        </is>
+      </c>
+      <c r="J668" t="inlineStr">
+        <is>
+          <t>2366</t>
+        </is>
+      </c>
+      <c r="K668" t="inlineStr">
+        <is>
+          <t>189</t>
+        </is>
+      </c>
+      <c r="L668" t="inlineStr">
+        <is>
+          <t>518</t>
+        </is>
+      </c>
+      <c r="M668" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="N668" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="O668" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="P668" t="inlineStr">
+        <is>
+          <t>['http://sns-webpic-qc.xhscdn.com/202602112040/77527399bb1401c02b909c91d6a45b20/1040g00831qa6dv9pga6g4a7r1e8cb33vmi8d66g!nd_dft_wlteh_jpg_3']</t>
+        </is>
+      </c>
+      <c r="Q668" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="R668" t="inlineStr">
+        <is>
+          <t>2025-12-20 12:31:29</t>
+        </is>
+      </c>
+      <c r="S668" t="inlineStr">
+        <is>
+          <t>未知</t>
+        </is>
+      </c>
+      <c r="T668" t="inlineStr">
+        <is>
+          <t>图1: OCR超时</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>6945e7e9000000000d03d348</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>https://www.xiaohongshu.com/explore/6945e7e9000000000d03d348?xsec_token=ABEi58ShmTcQxkgcxX0gUzNXSFkgGttjX6857ZKWzbJcQ=&amp;xsec_source=pc_user</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>图集</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>5b6150c56b58b741e26b8c7f</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>https://www.xiaohongshu.com/user/profile/5b6150c56b58b741e26b8c7f</t>
+        </is>
+      </c>
+      <c r="F669" t="inlineStr">
+        <is>
+          <t>还是叫吴富贵吧</t>
+        </is>
+      </c>
+      <c r="G669" t="inlineStr">
+        <is>
+          <t>https://sns-avatar-qc.xhscdn.com/avatar/1040g2jo31g9vkplp2s6g4a7r1e8cb33vdvgmpr0</t>
+        </is>
+      </c>
+      <c r="H669" t="inlineStr">
+        <is>
+          <t>好运一直眷顾你？ 呵呵 呵呵呵 呵呵呵呵</t>
+        </is>
+      </c>
+      <c r="I669" t="inlineStr">
+        <is>
+          <t>很奇怪的逻辑
+凭什么很多人就点点赞
+夸几句 不学习 不提高
+就可以心安理得的免费获取 你们以为的财富密码？
+人不是要靠自己吗？
+真把自己当天选之子了？
+什么我只要每年10％就满足了  说这话时 托下巴了吗</t>
+        </is>
+      </c>
+      <c r="J669" t="inlineStr">
+        <is>
+          <t>2606</t>
+        </is>
+      </c>
+      <c r="K669" t="inlineStr">
+        <is>
+          <t>198</t>
+        </is>
+      </c>
+      <c r="L669" t="inlineStr">
+        <is>
+          <t>737</t>
+        </is>
+      </c>
+      <c r="M669" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="N669" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="O669" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="P669" t="inlineStr">
+        <is>
+          <t>['http://sns-webpic-qc.xhscdn.com/202602112045/e02d2f07a3bbc1aa8d5de1ad7705f0d0/1040g00831q9ug5emga104a7r1e8cb33v4c35mp8!nd_dft_wlteh_jpg_3']</t>
+        </is>
+      </c>
+      <c r="Q669" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="R669" t="inlineStr">
+        <is>
+          <t>2025-12-20 08:03:53</t>
+        </is>
+      </c>
+      <c r="S669" t="inlineStr">
+        <is>
+          <t>未知</t>
+        </is>
+      </c>
+      <c r="T669" t="inlineStr">
+        <is>
+          <t>图1: OCR超时</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>6945e57b000000000d00f1e1</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>https://www.xiaohongshu.com/explore/6945e57b000000000d00f1e1?xsec_token=ABEi58ShmTcQxkgcxX0gUzNeEivOriL25rvHXBjHjdloA=&amp;xsec_source=pc_user</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>图集</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>5b6150c56b58b741e26b8c7f</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>https://www.xiaohongshu.com/user/profile/5b6150c56b58b741e26b8c7f</t>
+        </is>
+      </c>
+      <c r="F670" t="inlineStr">
+        <is>
+          <t>还是叫吴富贵吧</t>
+        </is>
+      </c>
+      <c r="G670" t="inlineStr">
+        <is>
+          <t>https://sns-avatar-qc.xhscdn.com/avatar/1040g2jo31g9vkplp2s6g4a7r1e8cb33vdvgmpr0</t>
+        </is>
+      </c>
+      <c r="H670" t="inlineStr">
+        <is>
+          <t>无标题</t>
+        </is>
+      </c>
+      <c r="I670" t="inlineStr">
+        <is>
+          <t>赠品＋业绩涨  A＋
+赠品＋业绩横  A-
+赠品＋业绩跌  B
+赠品＋ 业绩差 B-
+没赠品＋强成长B＋
+没赠品＋业绩横[汗颜R]
+没赠品＋业绩差[汗颜R][汗颜R][汗颜R]</t>
+        </is>
+      </c>
+      <c r="J670" t="inlineStr">
+        <is>
+          <t>2520</t>
+        </is>
+      </c>
+      <c r="K670" t="inlineStr">
+        <is>
+          <t>728</t>
+        </is>
+      </c>
+      <c r="L670" t="inlineStr">
+        <is>
+          <t>301</t>
+        </is>
+      </c>
+      <c r="M670" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="N670" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="O670" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="P670" t="inlineStr">
+        <is>
+          <t>['http://sns-webpic-qc.xhscdn.com/202602112051/a4acd970b7ad4f6e6d43050c3a9cb7a6/1040g00831q9ug5emga5g4a7r1e8cb33vv0u8ibg!nd_dft_wlteh_jpg_3']</t>
+        </is>
+      </c>
+      <c r="Q670" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="R670" t="inlineStr">
+        <is>
+          <t>2025-12-20 07:53:31</t>
+        </is>
+      </c>
+      <c r="S670" t="inlineStr">
+        <is>
+          <t>未知</t>
+        </is>
+      </c>
+      <c r="T670" t="inlineStr">
+        <is>
+          <t>图1: OCR超时</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>69457e15000000000d036f28</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>https://www.xiaohongshu.com/explore/69457e15000000000d036f28?xsec_token=ABEi58ShmTcQxkgcxX0gUzNTF4gNt0Dq1ykFdjK1t4uog=&amp;xsec_source=pc_user</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>图集</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>5b6150c56b58b741e26b8c7f</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>https://www.xiaohongshu.com/user/profile/5b6150c56b58b741e26b8c7f</t>
+        </is>
+      </c>
+      <c r="F671" t="inlineStr">
+        <is>
+          <t>还是叫吴富贵吧</t>
+        </is>
+      </c>
+      <c r="G671" t="inlineStr">
+        <is>
+          <t>https://sns-avatar-qc.xhscdn.com/avatar/1040g2jo31g9vkplp2s6g4a7r1e8cb33vdvgmpr0</t>
+        </is>
+      </c>
+      <c r="H671" t="inlineStr">
+        <is>
+          <t>一年啊又一年</t>
+        </is>
+      </c>
+      <c r="I671" t="inlineStr">
+        <is>
+          <t>2023年初是四大行
+2024年是股份制
+2025年是保险
+2026年是 券商＋变异电#我的炒股日记[话题]#</t>
+        </is>
+      </c>
+      <c r="J671" t="inlineStr">
+        <is>
+          <t>4078</t>
+        </is>
+      </c>
+      <c r="K671" t="inlineStr">
+        <is>
+          <t>1945</t>
+        </is>
+      </c>
+      <c r="L671" t="inlineStr">
+        <is>
+          <t>572</t>
+        </is>
+      </c>
+      <c r="M671" t="inlineStr">
+        <is>
+          <t>458</t>
+        </is>
+      </c>
+      <c r="N671" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="O671" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="P671" t="inlineStr">
+        <is>
+          <t>['http://sns-webpic-qc.xhscdn.com/202602112057/68778836ee53a9fb9968f64fc9594983/1040g00831q92gsko0a1g4a7r1e8cb33vbbtud9o!nd_dft_wlteh_jpg_3']</t>
+        </is>
+      </c>
+      <c r="Q671" t="inlineStr">
+        <is>
+          <t>['我的炒股日记']</t>
+        </is>
+      </c>
+      <c r="R671" t="inlineStr">
+        <is>
+          <t>2025-12-20 00:32:21</t>
+        </is>
+      </c>
+      <c r="S671" t="inlineStr">
+        <is>
+          <t>未知</t>
+        </is>
+      </c>
+      <c r="T671" t="inlineStr">
+        <is>
+          <t>图1: OCR超时</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>